<commit_message>
MSI: add btn_PopUpOk to pageRegConfirmationpopup (was only in pageHome); set Property=exists on all 11 verifyProperty steps missing it. Validated MSI 9->13
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/MSI/LSTP_MSI_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/MSI/LSTP_MSI_WF001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\MSI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751760E1-45F6-43D4-86C2-523A3A93D60D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1853219-0736-46CB-B646-CE81098F8647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{702FC42C-4FAC-40FC-8DEB-CEC87A00E4C0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{702FC42C-4FAC-40FC-8DEB-CEC87A00E4C0}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="266">
   <si>
     <t>StepNo</t>
   </si>
@@ -1638,6 +1638,9 @@
       <c r="F15" t="s">
         <v>31</v>
       </c>
+      <c r="G15" t="s">
+        <v>265</v>
+      </c>
       <c r="J15" t="b">
         <v>1</v>
       </c>
@@ -1771,6 +1774,9 @@
       <c r="F23" t="s">
         <v>31</v>
       </c>
+      <c r="G23" t="s">
+        <v>265</v>
+      </c>
       <c r="J23" t="b">
         <v>1</v>
       </c>
@@ -2055,6 +2061,9 @@
       <c r="F39" t="s">
         <v>31</v>
       </c>
+      <c r="G39" t="s">
+        <v>265</v>
+      </c>
       <c r="J39" t="b">
         <v>1</v>
       </c>
@@ -2395,6 +2404,9 @@
       <c r="F59" t="s">
         <v>31</v>
       </c>
+      <c r="G59" t="s">
+        <v>265</v>
+      </c>
       <c r="J59" t="b">
         <v>1</v>
       </c>
@@ -2638,6 +2650,9 @@
       <c r="F74" t="s">
         <v>31</v>
       </c>
+      <c r="G74" t="s">
+        <v>265</v>
+      </c>
       <c r="J74" t="b">
         <v>1</v>
       </c>
@@ -2689,6 +2704,9 @@
       <c r="F77" t="s">
         <v>31</v>
       </c>
+      <c r="G77" t="s">
+        <v>265</v>
+      </c>
       <c r="J77" t="b">
         <v>1</v>
       </c>
@@ -2757,6 +2775,9 @@
       <c r="F81" t="s">
         <v>31</v>
       </c>
+      <c r="G81" t="s">
+        <v>265</v>
+      </c>
       <c r="J81" t="b">
         <v>1</v>
       </c>
@@ -2952,6 +2973,9 @@
       <c r="F93" t="s">
         <v>31</v>
       </c>
+      <c r="G93" t="s">
+        <v>265</v>
+      </c>
       <c r="J93" t="b">
         <v>1</v>
       </c>
@@ -3003,6 +3027,9 @@
       <c r="F96" t="s">
         <v>31</v>
       </c>
+      <c r="G96" t="s">
+        <v>265</v>
+      </c>
       <c r="J96" t="b">
         <v>1</v>
       </c>
@@ -3071,6 +3098,9 @@
       <c r="F100" t="s">
         <v>31</v>
       </c>
+      <c r="G100" t="s">
+        <v>265</v>
+      </c>
       <c r="J100" t="b">
         <v>1</v>
       </c>
@@ -3152,6 +3182,9 @@
       </c>
       <c r="F105" t="s">
         <v>31</v>
+      </c>
+      <c r="G105" t="s">
+        <v>265</v>
       </c>
       <c r="J105" t="b">
         <v>1</v>

</xml_diff>